<commit_message>
Changed RetrieveComments and QueryTables API methods
The `sheetName` parameter now defaults to null and the first worksheet of the Excel workbook will be selected even if its name is not "Sheet1"
</commit_message>
<xml_diff>
--- a/tests/data/xlsx/TestQueryTable.xlsx
+++ b/tests/data/xlsx/TestQueryTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\computer\source\repos\MiniExcel\tests\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFDAFB0A-5F38-4F0F-8F4E-CDD99C681623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F41365-A010-4856-A516-A5D085020C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="1560" windowWidth="22755" windowHeight="11745" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30360" yWindow="1560" windowWidth="22755" windowHeight="11745" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>